<commit_message>
Align R27 system documents and add diagram component spreadsheet
</commit_message>
<xml_diff>
--- a/SYS/VENDING MACHINE GANTRY BILL OF MATERIALS - OFF THE SHELF COMPONENTS.xlsx
+++ b/SYS/VENDING MACHINE GANTRY BILL OF MATERIALS - OFF THE SHELF COMPONENTS.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vending Machine BOM" sheetId="1" r:id="R561557d953d04907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vending Machine BOM" sheetId="1" r:id="R666610fbf55b44aa"/>
   </x:sheets>
   <x:definedNames>
     <x:definedName name="COMM_TYPE">'Vending Machine BOM'!$F$1:$F$3</x:definedName>
@@ -13,9 +13,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t xml:space="preserve">BILL OF MATERIALS</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">PROJECT NAME:</x:t>
   </x:si>
   <x:si>
@@ -73,9 +70,6 @@
     <x:t xml:space="preserve">GANTRY AXIS</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">For Both X and Z-Axis</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">https://www.alibaba.com/product-detail/Nema-23-Closed-Loop-Stepper-Motor_1601462210871.html?spm=a2700.prosearch.normal_offer.d_title.70ab67afZCcPV5&amp;priceId=41e5753b040d4e17bc6bc6e0f8103217</x:t>
   </x:si>
   <x:si>
@@ -89,18 +83,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">https://www.alibaba.com/product-detail/EMTECH-Nema23-Planetary-Gearbox-3-10_1601689918939.html?spm=a2700.shop_plser.41413.5.1d8b4320viXRYQ</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">500W, 48V Power Supply  (For Stepper Motor)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">500W, 48V OUTPUT (ANY BRAND)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">S-500-48</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">For Nema23 Stepper Motor</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Slot Type Photosensor (Omron EE-SX674-WR or equivalent)</x:t>
@@ -332,7 +314,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -400,6 +382,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -616,589 +619,665 @@
   </x:cols>
   <x:sheetData>
     <x:row r="2">
-      <x:c r="D2" s="2" t="s">
-        <x:v>0</x:v>
+      <x:c r="D2" s="2" t="str">
+        <x:v>BILL OF MATERIALS - R27</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C4" t="s">
         <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" t="s">
-        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" t="s">
         <x:v>3</x:v>
-      </x:c>
-      <x:c r="C5" t="s">
-        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="15" customFormat="1" ht="15.75">
       <x:c r="A6" s="12" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="12" t="s">
+      <x:c r="C6" s="12" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="C6" s="12" t="s">
+      <x:c r="D6" s="12" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D6" s="12" t="s">
+      <x:c r="E6" s="13" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="E6" s="13" t="s">
+      <x:c r="F6" s="14" t="s">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="F6" s="14" t="s">
+      <x:c r="G6" s="14" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G6" s="14" t="s">
+      <x:c r="H6" s="14" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="H6" s="14" t="s">
+      <x:c r="I6" s="12" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="I6" s="12" t="s">
+      <x:c r="J6" s="12" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="J6" s="12" t="s">
+    </x:row>
+    <x:row r="7" s="11" customFormat="1" ht="80" customHeight="1">
+      <x:c r="A7" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B7" s="26">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C7" s="26"/>
+      <x:c r="D7" s="26" t="s">
         <x:v>14</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" s="11" customFormat="1">
-      <x:c r="A7" s="8">
+      <x:c r="E7" s="26" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F7" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G7" s="27" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="H7" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I7" s="26" t="str">
+        <x:v>X and Z; brake and driver supplied. Integrated/separate driver packaging, 24 V compatibility and input current TBC.</x:v>
+      </x:c>
+      <x:c r="J7" s="28" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" s="11" customFormat="1">
+      <x:c r="A8" s="26">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B8" s="26">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B7" s="8">
+      <x:c r="C8" s="26"/>
+      <x:c r="D8" s="26" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F8" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G8" s="27"/>
+      <x:c r="H8" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I8" s="26" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="J8" s="28" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" s="11" customFormat="1" ht="85" customHeight="1">
+      <x:c r="A9" s="26">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B9" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>Pc</x:v>
+      </x:c>
+      <x:c r="D9" s="26" t="str">
+        <x:v>24 V system power supply</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>24 V / 21 A / 504 W; capacity validation pending</x:v>
+      </x:c>
+      <x:c r="F9" s="27" t="str">
+        <x:v>SPECIAL PART</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>Mean Well RSP-500-24</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
+        <x:v>CABINET / ALL RAILS</x:v>
+      </x:c>
+      <x:c r="I9" s="26" t="str">
+        <x:v>Replaces superseded 48 V supply. Gantry operation at 24 V pending exact drive datasheet.</x:v>
+      </x:c>
+      <x:c r="J9" s="26" t="str">
+        <x:v>https://www.meanwell.com/Upload/PDF/RSP-500/RSP-500-SPEC.PDF</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" s="11" customFormat="1">
+      <x:c r="A10" s="26">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B10" s="26">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C10" s="26"/>
+      <x:c r="D10" s="26" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="E10" s="26" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F10" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G10" s="27" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="H10" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I10" s="26" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="J10" s="26"/>
+    </x:row>
+    <x:row r="11" s="11" customFormat="1">
+      <x:c r="A11" s="26">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B11" s="26">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C11" s="26"/>
+      <x:c r="D11" s="26" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="E11" s="26" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F11" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G11" s="27" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="H11" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I11" s="26" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="J11" s="26"/>
+    </x:row>
+    <x:row r="12" s="23" customFormat="1">
+      <x:c r="A12" s="29">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B12" s="29">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C12" s="29"/>
+      <x:c r="D12" s="29" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E12" s="29"/>
+      <x:c r="F12" s="30" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G12" s="30" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="H12" s="30" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="I12" s="29" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="J12" s="31" t="s">
+        <x:v>35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" s="11" customFormat="1">
+      <x:c r="A13" s="26">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B13" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C13" s="26"/>
+      <x:c r="D13" s="26" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="E13" s="26" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F13" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G13" s="27" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H13" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I13" s="26" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="J13" s="26" t="s">
+        <x:v>40</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" s="11" customFormat="1" ht="19.5" customHeight="1">
+      <x:c r="A14" s="26">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B14" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C14" s="26"/>
+      <x:c r="D14" s="26" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="F14" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G14" s="27" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="H14" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I14" s="26" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="J14" s="26"/>
+    </x:row>
+    <x:row r="15" s="11" customFormat="1">
+      <x:c r="A15" s="26">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B15" s="26">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C7" s="8"/>
-      <x:c r="D7" s="8" t="s">
+      <x:c r="C15" s="26" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D15" s="26" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E15" s="26" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="F15" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G15" s="27" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="H15" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I15" s="26" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="J15" s="28"/>
+    </x:row>
+    <x:row r="16" s="11" customFormat="1">
+      <x:c r="A16" s="26">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B16" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C16" s="26" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D16" s="26" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="E16" s="26" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="F16" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G16" s="27" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="H16" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I16" s="26" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="J16" s="26"/>
+    </x:row>
+    <x:row r="17" s="11" customFormat="1">
+      <x:c r="A17" s="26">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B17" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C17" s="26" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="D17" s="26" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="E17" s="26" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="F17" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G17" s="27" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="H17" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I17" s="26" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="J17" s="26"/>
+    </x:row>
+    <x:row r="18" s="11" customFormat="1">
+      <x:c r="A18" s="26">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B18" s="26">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C18" s="26" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="D18" s="32" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E18" s="26" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="F18" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G18" s="27" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="H18" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I18" s="26"/>
+      <x:c r="J18" s="26" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" s="11" customFormat="1" ht="30">
+      <x:c r="A19" s="26">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B19" s="26">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C19" s="26" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="D19" s="26" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="E19" s="26" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="F19" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G19" s="27" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="H19" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I19" s="26" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="J19" s="26" t="s">
+        <x:v>65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" s="11" customFormat="1" ht="30">
+      <x:c r="A20" s="26">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B20" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C20" s="26" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="D20" s="26" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="E20" s="26" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F20" s="27" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G20" s="27" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="H20" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I20" s="26" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="J20" s="26" t="s">
+        <x:v>71</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" s="11" customFormat="1" ht="30">
+      <x:c r="A21" s="26">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="s">
+      <x:c r="B21" s="26">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C21" s="26" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="D21" s="26" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="E21" s="26" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="F21" s="27" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F7" s="10" t="s">
+      <x:c r="G21" s="27" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="H21" s="27" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="I21" s="26" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="J21" s="26" t="s">
+        <x:v>75</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="78" customHeight="1">
+      <x:c r="A22" s="26" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B22" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C22" s="26" t="str">
+        <x:v>Pc</x:v>
+      </x:c>
+      <x:c r="D22" s="26" t="str">
+        <x:v>Ethernet panel-mount RJ45 adapter</x:v>
+      </x:c>
+      <x:c r="E22" s="26" t="str">
+        <x:v>Shielded Cat5e; RJ45 female × female; black plastic</x:v>
+      </x:c>
+      <x:c r="F22" s="27" t="str">
+        <x:v>STANDARD PART</x:v>
+      </x:c>
+      <x:c r="G22" s="27" t="str">
+        <x:v>1422N13</x:v>
+      </x:c>
+      <x:c r="H22" s="27" t="str">
+        <x:v>CABINET / NETWORK</x:v>
+      </x:c>
+      <x:c r="I22" s="26" t="str">
+        <x:v>McMaster-Carr; J2 rear panel; 0.95 in (24.13 mm) cutout; 0.14 in mounting holes; fasteners included</x:v>
+      </x:c>
+      <x:c r="J22" s="26" t="str">
+        <x:v>https://www.mcmaster.com/product/1422N13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="85" customHeight="1">
+      <x:c r="A23" s="26" t="n">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G7" s="10" t="s">
+      <x:c r="B23" s="26" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C23" s="26" t="str">
+        <x:v>Pcs</x:v>
+      </x:c>
+      <x:c r="D23" s="26" t="str">
+        <x:v>LANECTRL front metal bracket</x:v>
+      </x:c>
+      <x:c r="E23" s="26" t="str">
+        <x:v>Per user-supplied DWG; PCB fit not yet verified</x:v>
+      </x:c>
+      <x:c r="F23" s="27" t="str">
+        <x:v>CUSTOM PART</x:v>
+      </x:c>
+      <x:c r="G23" s="27" t="str">
+        <x:v>LANE DRAWING SPACE FOR UMIT.DWG</x:v>
+      </x:c>
+      <x:c r="H23" s="27" t="str">
+        <x:v>LANE ROWS</x:v>
+      </x:c>
+      <x:c r="I23" s="26" t="str">
+        <x:v>One per row assumed; confirm drawing quantity and button/LED clearances.</x:v>
+      </x:c>
+      <x:c r="J23" s="26" t="str">
+        <x:v>../MEC/01_CAD_MODELS/LANE DRAWING SPACE FOR UMIT.DWG</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="85" customHeight="1">
+      <x:c r="A24" s="26" t="n">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="H7" s="10" t="s">
+      <x:c r="B24" s="26" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C24" s="26" t="str">
+        <x:v>Pcs</x:v>
+      </x:c>
+      <x:c r="D24" s="26" t="str">
+        <x:v>Conveyor assembly with DC motor</x:v>
+      </x:c>
+      <x:c r="E24" s="26" t="str">
+        <x:v>24 V; &lt;=0.2 A no-load; 5.8 cm/s; &lt;=6 kg</x:v>
+      </x:c>
+      <x:c r="F24" s="27" t="str">
+        <x:v>SPECIAL PART</x:v>
+      </x:c>
+      <x:c r="G24" s="27" t="str">
+        <x:v>CB002-24V-573mm</x:v>
+      </x:c>
+      <x:c r="H24" s="27" t="str">
+        <x:v>LANE ROWS</x:v>
+      </x:c>
+      <x:c r="I24" s="26" t="str">
+        <x:v>Loaded/stall current, signal reference and reversal compatibility remain open.</x:v>
+      </x:c>
+      <x:c r="J24" s="26" t="str">
+        <x:v>Conveyor belt(CB002-24V-573mm).pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="85" customHeight="1">
+      <x:c r="A25" s="26" t="n">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="I7" s="8" t="s">
+      <x:c r="B25" s="26" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C25" s="26" t="str">
+        <x:v>Set</x:v>
+      </x:c>
+      <x:c r="D25" s="26" t="str">
+        <x:v>Electrical controllers, wiring and protection</x:v>
+      </x:c>
+      <x:c r="E25" s="26" t="str">
+        <x:v>Authoritative quantities and selections in electrical workbook</x:v>
+      </x:c>
+      <x:c r="F25" s="27" t="str">
+        <x:v>REFERENCE</x:v>
+      </x:c>
+      <x:c r="G25" s="27" t="str">
+        <x:v>APDU_Electrical_Tables_R27.xlsx</x:v>
+      </x:c>
+      <x:c r="H25" s="27" t="str">
+        <x:v>SYSTEM</x:v>
+      </x:c>
+      <x:c r="I25" s="26" t="str">
+        <x:v>Reference only: use BOM/PCBs/Connectors/Cables/Fuses sheets; do not duplicate purchase lines.</x:v>
+      </x:c>
+      <x:c r="J25" s="26" t="str">
+        <x:v>APDU_Electrical_Tables_R27.xlsx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="85" customHeight="1">
+      <x:c r="A26" s="26" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="J7" s="18" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" s="11" customFormat="1">
-      <x:c r="A8" s="8">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B8" s="8">
+      <x:c r="B26" s="26" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="8"/>
-      <x:c r="D8" s="8" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="E8" s="9" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="F8" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G8" s="10"/>
-      <x:c r="H8" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I8" s="8" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="J8" s="18" t="s">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" s="11" customFormat="1">
-      <x:c r="A9" s="8">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B9" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C9" s="8"/>
-      <x:c r="D9" s="8" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="E9" s="9" t="s">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="F9" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G9" s="10" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="H9" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I9" s="8" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="J9" s="8"/>
-    </x:row>
-    <x:row r="10" s="11" customFormat="1">
-      <x:c r="A10" s="8">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B10" s="8">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C10" s="8"/>
-      <x:c r="D10" s="8" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="E10" s="9" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F10" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G10" s="10" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="H10" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I10" s="9" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="J10" s="8"/>
-    </x:row>
-    <x:row r="11" s="11" customFormat="1">
-      <x:c r="A11" s="8">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B11" s="8">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C11" s="8"/>
-      <x:c r="D11" s="8" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="E11" s="9" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="F11" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G11" s="10" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H11" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I11" s="9" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="J11" s="8"/>
-    </x:row>
-    <x:row r="12" s="23" customFormat="1">
-      <x:c r="A12" s="19">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="B12" s="19">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C12" s="19"/>
-      <x:c r="D12" s="19" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="E12" s="20"/>
-      <x:c r="F12" s="21" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G12" s="21" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="H12" s="21" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="I12" s="19" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="J12" s="22" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" s="11" customFormat="1">
-      <x:c r="A13" s="8">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B13" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C13" s="8"/>
-      <x:c r="D13" s="8" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E13" s="9" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="F13" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G13" s="10" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="H13" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I13" s="8" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="J13" s="8" t="s">
-        <x:v>46</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" s="11" customFormat="1" ht="19.5" customHeight="1">
-      <x:c r="A14" s="8">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="B14" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C14" s="8"/>
-      <x:c r="D14" s="8" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="E14" s="9" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="F14" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G14" s="10" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="H14" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I14" s="8" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="J14" s="8"/>
-    </x:row>
-    <x:row r="15" s="11" customFormat="1">
-      <x:c r="A15" s="8">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B15" s="8">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C15" s="8" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D15" s="8" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E15" s="9" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="F15" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G15" s="10" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="H15" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I15" s="8" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J15" s="18"/>
-    </x:row>
-    <x:row r="16" s="11" customFormat="1">
-      <x:c r="A16" s="8">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B16" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C16" s="8" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D16" s="8" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="F16" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G16" s="10" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="H16" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I16" s="8" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J16" s="8"/>
-    </x:row>
-    <x:row r="17" s="11" customFormat="1">
-      <x:c r="A17" s="8">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="B17" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C17" s="8" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="D17" s="8" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="E17" s="9" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="F17" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G17" s="10" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="H17" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I17" s="8" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="J17" s="8"/>
-    </x:row>
-    <x:row r="18" s="11" customFormat="1">
-      <x:c r="A18" s="8">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B18" s="8">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="D18" s="17" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E18" s="9" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F18" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G18" s="10" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="H18" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I18" s="8"/>
-      <x:c r="J18" s="8" t="s">
-        <x:v>66</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" s="11" customFormat="1" ht="30">
-      <x:c r="A19" s="8">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="B19" s="8">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C19" s="8" t="s">
-        <x:v>62</x:v>
-      </x:c>
-      <x:c r="D19" s="8" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="E19" s="9" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="F19" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G19" s="10" t="s">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="H19" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I19" s="8" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="J19" s="8" t="s">
-        <x:v>71</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" s="11" customFormat="1" ht="30">
-      <x:c r="A20" s="8">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B20" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C20" s="8" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="D20" s="8" t="s">
-        <x:v>73</x:v>
-      </x:c>
-      <x:c r="E20" s="9" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="F20" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G20" s="10" t="s">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="H20" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I20" s="9" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="J20" s="8" t="s">
-        <x:v>77</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" s="11" customFormat="1" ht="30">
-      <x:c r="A21" s="8">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B21" s="8">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C21" s="8" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="D21" s="8" t="s">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E21" s="9" t="s">
-        <x:v>74</x:v>
-      </x:c>
-      <x:c r="F21" s="10" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="G21" s="10" t="s">
-        <x:v>79</x:v>
-      </x:c>
-      <x:c r="H21" s="10" t="s">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I21" s="9" t="s">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="J21" s="8" t="s">
-        <x:v>81</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="78" customHeight="1">
-      <x:c r="A22" s="24" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B22" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C22" s="24" t="str">
-        <x:v>Pc</x:v>
-      </x:c>
-      <x:c r="D22" s="24" t="str">
-        <x:v>Ethernet panel-mount RJ45 adapter</x:v>
-      </x:c>
-      <x:c r="E22" s="24" t="str">
-        <x:v>Shielded Cat5e; RJ45 female × female; black plastic</x:v>
-      </x:c>
-      <x:c r="F22" s="25" t="str">
-        <x:v>STANDARD PART</x:v>
-      </x:c>
-      <x:c r="G22" s="25" t="str">
-        <x:v>1422N13</x:v>
-      </x:c>
-      <x:c r="H22" s="25" t="str">
-        <x:v>CABINET / NETWORK</x:v>
-      </x:c>
-      <x:c r="I22" s="24" t="str">
-        <x:v>McMaster-Carr; J2 rear panel; 0.95 in (24.13 mm) cutout; 0.14 in mounting holes; fasteners included</x:v>
-      </x:c>
-      <x:c r="J22" s="24" t="str">
-        <x:v>https://www.mcmaster.com/product/1422N13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="13.5" customHeight="1">
-      <x:c r="A23" s="3">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="B23" s="3"/>
-      <x:c r="C23" s="3"/>
-      <x:c r="D23" s="3"/>
-      <x:c r="E23" s="5"/>
-      <x:c r="F23" s="4"/>
-      <x:c r="G23" s="4"/>
-      <x:c r="H23" s="4"/>
-      <x:c r="I23" s="3"/>
-      <x:c r="J23" s="3"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="3">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B24" s="3"/>
-      <x:c r="C24" s="3"/>
-      <x:c r="D24" s="3"/>
-      <x:c r="E24" s="5"/>
-      <x:c r="F24" s="4"/>
-      <x:c r="G24" s="4"/>
-      <x:c r="H24" s="4"/>
-      <x:c r="I24" s="3"/>
-      <x:c r="J24" s="3"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="3">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="B25" s="3"/>
-      <x:c r="C25" s="3"/>
-      <x:c r="D25" s="3"/>
-      <x:c r="E25" s="5"/>
-      <x:c r="F25" s="4"/>
-      <x:c r="G25" s="4"/>
-      <x:c r="H25" s="4"/>
-      <x:c r="I25" s="3"/>
-      <x:c r="J25" s="3"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="3">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B26" s="3"/>
-      <x:c r="C26" s="3"/>
-      <x:c r="D26" s="3"/>
-      <x:c r="E26" s="5"/>
-      <x:c r="F26" s="4"/>
-      <x:c r="G26" s="4"/>
-      <x:c r="H26" s="4"/>
-      <x:c r="I26" s="3"/>
-      <x:c r="J26" s="3"/>
+      <x:c r="C26" s="26" t="str">
+        <x:v>Set</x:v>
+      </x:c>
+      <x:c r="D26" s="26" t="str">
+        <x:v>Labeling mechanism parts</x:v>
+      </x:c>
+      <x:c r="E26" s="26" t="str">
+        <x:v>Chuck/jaw motors, servo, sensor and marker require selection confirmation</x:v>
+      </x:c>
+      <x:c r="F26" s="27" t="str">
+        <x:v>REFERENCE</x:v>
+      </x:c>
+      <x:c r="G26" s="27" t="str">
+        <x:v>See electrical BOM and OpenItems O10/O11</x:v>
+      </x:c>
+      <x:c r="H26" s="27" t="str">
+        <x:v>LABELING</x:v>
+      </x:c>
+      <x:c r="I26" s="26" t="str">
+        <x:v>Reference only; unresolved MPNs and marker power prevent purchase release.</x:v>
+      </x:c>
+      <x:c r="J26" s="26" t="str">
+        <x:v>APDU_Electrical_Tables_R27.xlsx</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="3">
@@ -2271,9 +2350,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="R4a3984d95b184401"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="Rec1877dc4d76436a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="R0fe9430486c04fb9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="R741cd5faa18749d6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" r:id="R70b2002943764675"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" r:id="R04be1771b0994286"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>